<commit_message>
Add EDI Compare page: week-by-week changes between two EDI files
Sample data now has four weekly EDI files with deliberate changes, and the
generator sets each file's creation time to its send date (EDI pages order by it).
</commit_message>
<xml_diff>
--- a/sample_data/edi/EDI_VW_SAMPLE_20261009.xlsx
+++ b/sample_data/edi/EDI_VW_SAMPLE_20261009.xlsx
@@ -459,7 +459,7 @@
         <v>46297</v>
       </c>
       <c r="C2" t="n">
-        <v>1369</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="3">
@@ -472,7 +472,7 @@
         <v>46298</v>
       </c>
       <c r="C3" t="n">
-        <v>1363</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="4">
@@ -485,7 +485,7 @@
         <v>46300</v>
       </c>
       <c r="C4" t="n">
-        <v>1376</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="5">
@@ -498,7 +498,7 @@
         <v>46301</v>
       </c>
       <c r="C5" t="n">
-        <v>1547</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="6">
@@ -511,7 +511,7 @@
         <v>46302</v>
       </c>
       <c r="C6" t="n">
-        <v>1373</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="7">
@@ -524,7 +524,7 @@
         <v>46303</v>
       </c>
       <c r="C7" t="n">
-        <v>1085</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="8">
@@ -537,7 +537,7 @@
         <v>46304</v>
       </c>
       <c r="C8" t="n">
-        <v>1469</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="9">
@@ -550,7 +550,7 @@
         <v>46305</v>
       </c>
       <c r="C9" t="n">
-        <v>1343</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="10">
@@ -563,7 +563,7 @@
         <v>46307</v>
       </c>
       <c r="C10" t="n">
-        <v>1354</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="11">
@@ -576,7 +576,7 @@
         <v>46308</v>
       </c>
       <c r="C11" t="n">
-        <v>1424</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="12">
@@ -589,7 +589,7 @@
         <v>46309</v>
       </c>
       <c r="C12" t="n">
-        <v>1448</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="13">
@@ -602,7 +602,7 @@
         <v>46310</v>
       </c>
       <c r="C13" t="n">
-        <v>1644</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="14">
@@ -615,7 +615,7 @@
         <v>46311</v>
       </c>
       <c r="C14" t="n">
-        <v>1537</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="15">
@@ -628,7 +628,7 @@
         <v>46312</v>
       </c>
       <c r="C15" t="n">
-        <v>1423</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="16">
@@ -641,7 +641,7 @@
         <v>46314</v>
       </c>
       <c r="C16" t="n">
-        <v>1244</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="17">
@@ -654,7 +654,7 @@
         <v>46315</v>
       </c>
       <c r="C17" t="n">
-        <v>1186</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="18">
@@ -667,7 +667,7 @@
         <v>46316</v>
       </c>
       <c r="C18" t="n">
-        <v>1451</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="19">
@@ -680,7 +680,7 @@
         <v>46317</v>
       </c>
       <c r="C19" t="n">
-        <v>1675</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="20">
@@ -693,7 +693,7 @@
         <v>46318</v>
       </c>
       <c r="C20" t="n">
-        <v>1408</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="21">
@@ -706,7 +706,7 @@
         <v>46319</v>
       </c>
       <c r="C21" t="n">
-        <v>1377</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="22">
@@ -719,7 +719,7 @@
         <v>46321</v>
       </c>
       <c r="C22" t="n">
-        <v>1511</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="23">
@@ -732,7 +732,7 @@
         <v>46322</v>
       </c>
       <c r="C23" t="n">
-        <v>1094</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="24">
@@ -745,7 +745,7 @@
         <v>46323</v>
       </c>
       <c r="C24" t="n">
-        <v>1334</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="25">
@@ -758,7 +758,7 @@
         <v>46324</v>
       </c>
       <c r="C25" t="n">
-        <v>1502</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="26">
@@ -771,7 +771,7 @@
         <v>46325</v>
       </c>
       <c r="C26" t="n">
-        <v>1583</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="27">
@@ -784,7 +784,7 @@
         <v>46326</v>
       </c>
       <c r="C27" t="n">
-        <v>1349</v>
+        <v>931</v>
       </c>
     </row>
     <row r="28">
@@ -797,7 +797,7 @@
         <v>46328</v>
       </c>
       <c r="C28" t="n">
-        <v>1479</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="29">
@@ -810,7 +810,7 @@
         <v>46329</v>
       </c>
       <c r="C29" t="n">
-        <v>1452</v>
+        <v>836</v>
       </c>
     </row>
     <row r="30">
@@ -823,7 +823,7 @@
         <v>46330</v>
       </c>
       <c r="C30" t="n">
-        <v>1564</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="31">
@@ -836,7 +836,7 @@
         <v>46331</v>
       </c>
       <c r="C31" t="n">
-        <v>1166</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="32">
@@ -849,7 +849,7 @@
         <v>46332</v>
       </c>
       <c r="C32" t="n">
-        <v>1519</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="33">
@@ -862,7 +862,7 @@
         <v>46333</v>
       </c>
       <c r="C33" t="n">
-        <v>1081</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="34">
@@ -875,7 +875,7 @@
         <v>46335</v>
       </c>
       <c r="C34" t="n">
-        <v>849</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="35">
@@ -888,7 +888,7 @@
         <v>46336</v>
       </c>
       <c r="C35" t="n">
-        <v>1272</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="36">
@@ -901,7 +901,7 @@
         <v>46337</v>
       </c>
       <c r="C36" t="n">
-        <v>1207</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="37">
@@ -914,7 +914,7 @@
         <v>46338</v>
       </c>
       <c r="C37" t="n">
-        <v>1583</v>
+        <v>1612</v>
       </c>
     </row>
     <row r="38">
@@ -927,7 +927,7 @@
         <v>46339</v>
       </c>
       <c r="C38" t="n">
-        <v>1539</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="39">
@@ -940,7 +940,7 @@
         <v>46340</v>
       </c>
       <c r="C39" t="n">
-        <v>1143</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="40">
@@ -953,7 +953,7 @@
         <v>46342</v>
       </c>
       <c r="C40" t="n">
-        <v>1577</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="41">
@@ -966,7 +966,7 @@
         <v>46343</v>
       </c>
       <c r="C41" t="n">
-        <v>1189</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="42">
@@ -979,7 +979,7 @@
         <v>46344</v>
       </c>
       <c r="C42" t="n">
-        <v>1381</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="43">
@@ -992,7 +992,7 @@
         <v>46345</v>
       </c>
       <c r="C43" t="n">
-        <v>1338</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="44">
@@ -1005,7 +1005,7 @@
         <v>46346</v>
       </c>
       <c r="C44" t="n">
-        <v>1424</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="45">
@@ -1018,7 +1018,7 @@
         <v>46347</v>
       </c>
       <c r="C45" t="n">
-        <v>1571</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="46">
@@ -1031,7 +1031,7 @@
         <v>46349</v>
       </c>
       <c r="C46" t="n">
-        <v>1534</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="47">
@@ -1044,7 +1044,7 @@
         <v>46350</v>
       </c>
       <c r="C47" t="n">
-        <v>1473</v>
+        <v>979</v>
       </c>
     </row>
     <row r="48">
@@ -1057,7 +1057,7 @@
         <v>46351</v>
       </c>
       <c r="C48" t="n">
-        <v>1536</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="49">
@@ -1070,7 +1070,7 @@
         <v>46352</v>
       </c>
       <c r="C49" t="n">
-        <v>1500</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="50">
@@ -1083,7 +1083,7 @@
         <v>46353</v>
       </c>
       <c r="C50" t="n">
-        <v>1268</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="51">
@@ -1096,7 +1096,7 @@
         <v>46354</v>
       </c>
       <c r="C51" t="n">
-        <v>1249</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="52">
@@ -1109,7 +1109,7 @@
         <v>46356</v>
       </c>
       <c r="C52" t="n">
-        <v>1301</v>
+        <v>855</v>
       </c>
     </row>
     <row r="53">
@@ -1122,7 +1122,7 @@
         <v>46357</v>
       </c>
       <c r="C53" t="n">
-        <v>1504</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="54">
@@ -1135,7 +1135,7 @@
         <v>46358</v>
       </c>
       <c r="C54" t="n">
-        <v>1347</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="55">
@@ -1148,7 +1148,7 @@
         <v>46359</v>
       </c>
       <c r="C55" t="n">
-        <v>1890</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="56">
@@ -1161,7 +1161,7 @@
         <v>46360</v>
       </c>
       <c r="C56" t="n">
-        <v>1227</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="57">
@@ -1174,7 +1174,7 @@
         <v>46361</v>
       </c>
       <c r="C57" t="n">
-        <v>1169</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="58">
@@ -1187,7 +1187,7 @@
         <v>46363</v>
       </c>
       <c r="C58" t="n">
-        <v>1561</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="59">
@@ -1200,7 +1200,7 @@
         <v>46364</v>
       </c>
       <c r="C59" t="n">
-        <v>1698</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="60">
@@ -1213,7 +1213,7 @@
         <v>46365</v>
       </c>
       <c r="C60" t="n">
-        <v>1506</v>
+        <v>1737</v>
       </c>
     </row>
     <row r="61">
@@ -1226,7 +1226,7 @@
         <v>46366</v>
       </c>
       <c r="C61" t="n">
-        <v>1575</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="62">
@@ -1239,7 +1239,7 @@
         <v>46297</v>
       </c>
       <c r="C62" t="n">
-        <v>789</v>
+        <v>635</v>
       </c>
     </row>
     <row r="63">
@@ -1252,7 +1252,7 @@
         <v>46298</v>
       </c>
       <c r="C63" t="n">
-        <v>640</v>
+        <v>624</v>
       </c>
     </row>
     <row r="64">
@@ -1265,7 +1265,7 @@
         <v>46300</v>
       </c>
       <c r="C64" t="n">
-        <v>511</v>
+        <v>557</v>
       </c>
     </row>
     <row r="65">
@@ -1278,7 +1278,7 @@
         <v>46301</v>
       </c>
       <c r="C65" t="n">
-        <v>598</v>
+        <v>773</v>
       </c>
     </row>
     <row r="66">
@@ -1291,7 +1291,7 @@
         <v>46302</v>
       </c>
       <c r="C66" t="n">
-        <v>742</v>
+        <v>524</v>
       </c>
     </row>
     <row r="67">
@@ -1304,7 +1304,7 @@
         <v>46303</v>
       </c>
       <c r="C67" t="n">
-        <v>509</v>
+        <v>583</v>
       </c>
     </row>
     <row r="68">
@@ -1317,7 +1317,7 @@
         <v>46304</v>
       </c>
       <c r="C68" t="n">
-        <v>653</v>
+        <v>703</v>
       </c>
     </row>
     <row r="69">
@@ -1330,7 +1330,7 @@
         <v>46305</v>
       </c>
       <c r="C69" t="n">
-        <v>674</v>
+        <v>765</v>
       </c>
     </row>
     <row r="70">
@@ -1343,7 +1343,7 @@
         <v>46307</v>
       </c>
       <c r="C70" t="n">
-        <v>619</v>
+        <v>680</v>
       </c>
     </row>
     <row r="71">
@@ -1356,7 +1356,7 @@
         <v>46308</v>
       </c>
       <c r="C71" t="n">
-        <v>720</v>
+        <v>670</v>
       </c>
     </row>
     <row r="72">
@@ -1369,7 +1369,7 @@
         <v>46309</v>
       </c>
       <c r="C72" t="n">
-        <v>706</v>
+        <v>654</v>
       </c>
     </row>
     <row r="73">
@@ -1382,7 +1382,7 @@
         <v>46310</v>
       </c>
       <c r="C73" t="n">
-        <v>876</v>
+        <v>719</v>
       </c>
     </row>
     <row r="74">
@@ -1395,7 +1395,7 @@
         <v>46311</v>
       </c>
       <c r="C74" t="n">
-        <v>710</v>
+        <v>629</v>
       </c>
     </row>
     <row r="75">
@@ -1408,7 +1408,7 @@
         <v>46312</v>
       </c>
       <c r="C75" t="n">
-        <v>590</v>
+        <v>665</v>
       </c>
     </row>
     <row r="76">
@@ -1421,7 +1421,7 @@
         <v>46314</v>
       </c>
       <c r="C76" t="n">
-        <v>595</v>
+        <v>644</v>
       </c>
     </row>
     <row r="77">
@@ -1434,7 +1434,7 @@
         <v>46315</v>
       </c>
       <c r="C77" t="n">
-        <v>568</v>
+        <v>721</v>
       </c>
     </row>
     <row r="78">
@@ -1447,7 +1447,7 @@
         <v>46316</v>
       </c>
       <c r="C78" t="n">
-        <v>742</v>
+        <v>691</v>
       </c>
     </row>
     <row r="79">
@@ -1460,7 +1460,7 @@
         <v>46317</v>
       </c>
       <c r="C79" t="n">
-        <v>594</v>
+        <v>843</v>
       </c>
     </row>
     <row r="80">
@@ -1473,7 +1473,7 @@
         <v>46318</v>
       </c>
       <c r="C80" t="n">
-        <v>643</v>
+        <v>679</v>
       </c>
     </row>
     <row r="81">
@@ -1486,7 +1486,7 @@
         <v>46319</v>
       </c>
       <c r="C81" t="n">
-        <v>723</v>
+        <v>613</v>
       </c>
     </row>
     <row r="82">
@@ -1499,7 +1499,7 @@
         <v>46321</v>
       </c>
       <c r="C82" t="n">
-        <v>579</v>
+        <v>644</v>
       </c>
     </row>
     <row r="83">
@@ -1512,7 +1512,7 @@
         <v>46322</v>
       </c>
       <c r="C83" t="n">
-        <v>621</v>
+        <v>733</v>
       </c>
     </row>
     <row r="84">
@@ -1525,7 +1525,7 @@
         <v>46323</v>
       </c>
       <c r="C84" t="n">
-        <v>470</v>
+        <v>610</v>
       </c>
     </row>
     <row r="85">
@@ -1538,7 +1538,7 @@
         <v>46324</v>
       </c>
       <c r="C85" t="n">
-        <v>544</v>
+        <v>694</v>
       </c>
     </row>
     <row r="86">
@@ -1551,7 +1551,7 @@
         <v>46325</v>
       </c>
       <c r="C86" t="n">
-        <v>594</v>
+        <v>843</v>
       </c>
     </row>
     <row r="87">
@@ -1564,7 +1564,7 @@
         <v>46326</v>
       </c>
       <c r="C87" t="n">
-        <v>690</v>
+        <v>400</v>
       </c>
     </row>
     <row r="88">
@@ -1577,7 +1577,7 @@
         <v>46328</v>
       </c>
       <c r="C88" t="n">
-        <v>766</v>
+        <v>666</v>
       </c>
     </row>
     <row r="89">
@@ -1590,7 +1590,7 @@
         <v>46329</v>
       </c>
       <c r="C89" t="n">
-        <v>648</v>
+        <v>697</v>
       </c>
     </row>
     <row r="90">
@@ -1603,7 +1603,7 @@
         <v>46330</v>
       </c>
       <c r="C90" t="n">
-        <v>675</v>
+        <v>670</v>
       </c>
     </row>
     <row r="91">
@@ -1616,7 +1616,7 @@
         <v>46331</v>
       </c>
       <c r="C91" t="n">
-        <v>666</v>
+        <v>600</v>
       </c>
     </row>
     <row r="92">
@@ -1629,7 +1629,7 @@
         <v>46332</v>
       </c>
       <c r="C92" t="n">
-        <v>755</v>
+        <v>703</v>
       </c>
     </row>
     <row r="93">
@@ -1642,7 +1642,7 @@
         <v>46333</v>
       </c>
       <c r="C93" t="n">
-        <v>737</v>
+        <v>685</v>
       </c>
     </row>
     <row r="94">
@@ -1655,7 +1655,7 @@
         <v>46335</v>
       </c>
       <c r="C94" t="n">
-        <v>676</v>
+        <v>897</v>
       </c>
     </row>
     <row r="95">
@@ -1668,7 +1668,7 @@
         <v>46336</v>
       </c>
       <c r="C95" t="n">
-        <v>551</v>
+        <v>688</v>
       </c>
     </row>
     <row r="96">
@@ -1681,7 +1681,7 @@
         <v>46337</v>
       </c>
       <c r="C96" t="n">
-        <v>738</v>
+        <v>595</v>
       </c>
     </row>
     <row r="97">
@@ -1694,7 +1694,7 @@
         <v>46338</v>
       </c>
       <c r="C97" t="n">
-        <v>687</v>
+        <v>641</v>
       </c>
     </row>
     <row r="98">
@@ -1707,7 +1707,7 @@
         <v>46339</v>
       </c>
       <c r="C98" t="n">
-        <v>769</v>
+        <v>621</v>
       </c>
     </row>
     <row r="99">
@@ -1720,7 +1720,7 @@
         <v>46340</v>
       </c>
       <c r="C99" t="n">
-        <v>647</v>
+        <v>655</v>
       </c>
     </row>
     <row r="100">
@@ -1733,7 +1733,7 @@
         <v>46342</v>
       </c>
       <c r="C100" t="n">
-        <v>840</v>
+        <v>598</v>
       </c>
     </row>
     <row r="101">
@@ -1746,7 +1746,7 @@
         <v>46343</v>
       </c>
       <c r="C101" t="n">
-        <v>615</v>
+        <v>752</v>
       </c>
     </row>
     <row r="102">
@@ -1759,7 +1759,7 @@
         <v>46344</v>
       </c>
       <c r="C102" t="n">
-        <v>805</v>
+        <v>542</v>
       </c>
     </row>
     <row r="103">
@@ -1772,7 +1772,7 @@
         <v>46345</v>
       </c>
       <c r="C103" t="n">
-        <v>661</v>
+        <v>651</v>
       </c>
     </row>
     <row r="104">
@@ -1785,7 +1785,7 @@
         <v>46346</v>
       </c>
       <c r="C104" t="n">
-        <v>599</v>
+        <v>742</v>
       </c>
     </row>
     <row r="105">
@@ -1798,7 +1798,7 @@
         <v>46347</v>
       </c>
       <c r="C105" t="n">
-        <v>539</v>
+        <v>727</v>
       </c>
     </row>
     <row r="106">
@@ -1811,7 +1811,7 @@
         <v>46349</v>
       </c>
       <c r="C106" t="n">
-        <v>635</v>
+        <v>485</v>
       </c>
     </row>
     <row r="107">
@@ -1824,7 +1824,7 @@
         <v>46350</v>
       </c>
       <c r="C107" t="n">
-        <v>788</v>
+        <v>606</v>
       </c>
     </row>
     <row r="108">
@@ -1837,7 +1837,7 @@
         <v>46351</v>
       </c>
       <c r="C108" t="n">
-        <v>729</v>
+        <v>624</v>
       </c>
     </row>
     <row r="109">
@@ -1850,7 +1850,7 @@
         <v>46352</v>
       </c>
       <c r="C109" t="n">
-        <v>717</v>
+        <v>706</v>
       </c>
     </row>
     <row r="110">
@@ -1863,7 +1863,7 @@
         <v>46353</v>
       </c>
       <c r="C110" t="n">
-        <v>418</v>
+        <v>767</v>
       </c>
     </row>
     <row r="111">
@@ -1876,7 +1876,7 @@
         <v>46354</v>
       </c>
       <c r="C111" t="n">
-        <v>719</v>
+        <v>384</v>
       </c>
     </row>
     <row r="112">
@@ -1889,7 +1889,7 @@
         <v>46356</v>
       </c>
       <c r="C112" t="n">
-        <v>704</v>
+        <v>506</v>
       </c>
     </row>
     <row r="113">
@@ -1902,7 +1902,7 @@
         <v>46357</v>
       </c>
       <c r="C113" t="n">
-        <v>596</v>
+        <v>709</v>
       </c>
     </row>
     <row r="114">
@@ -1915,7 +1915,7 @@
         <v>46358</v>
       </c>
       <c r="C114" t="n">
-        <v>588</v>
+        <v>503</v>
       </c>
     </row>
     <row r="115">
@@ -1928,7 +1928,7 @@
         <v>46359</v>
       </c>
       <c r="C115" t="n">
-        <v>649</v>
+        <v>658</v>
       </c>
     </row>
     <row r="116">
@@ -1941,7 +1941,7 @@
         <v>46360</v>
       </c>
       <c r="C116" t="n">
-        <v>818</v>
+        <v>751</v>
       </c>
     </row>
     <row r="117">
@@ -1954,7 +1954,7 @@
         <v>46361</v>
       </c>
       <c r="C117" t="n">
-        <v>547</v>
+        <v>641</v>
       </c>
     </row>
     <row r="118">
@@ -1967,7 +1967,7 @@
         <v>46363</v>
       </c>
       <c r="C118" t="n">
-        <v>608</v>
+        <v>721</v>
       </c>
     </row>
     <row r="119">
@@ -1980,7 +1980,7 @@
         <v>46364</v>
       </c>
       <c r="C119" t="n">
-        <v>782</v>
+        <v>657</v>
       </c>
     </row>
     <row r="120">
@@ -1993,7 +1993,7 @@
         <v>46365</v>
       </c>
       <c r="C120" t="n">
-        <v>606</v>
+        <v>636</v>
       </c>
     </row>
     <row r="121">
@@ -2006,7 +2006,7 @@
         <v>46366</v>
       </c>
       <c r="C121" t="n">
-        <v>614</v>
+        <v>798</v>
       </c>
     </row>
     <row r="122">
@@ -2019,7 +2019,7 @@
         <v>46297</v>
       </c>
       <c r="C122" t="n">
-        <v>913</v>
+        <v>884</v>
       </c>
     </row>
     <row r="123">
@@ -2032,7 +2032,7 @@
         <v>46298</v>
       </c>
       <c r="C123" t="n">
-        <v>732</v>
+        <v>823</v>
       </c>
     </row>
     <row r="124">
@@ -2045,7 +2045,7 @@
         <v>46300</v>
       </c>
       <c r="C124" t="n">
-        <v>929</v>
+        <v>961</v>
       </c>
     </row>
     <row r="125">
@@ -2058,7 +2058,7 @@
         <v>46301</v>
       </c>
       <c r="C125" t="n">
-        <v>736</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="126">
@@ -2071,7 +2071,7 @@
         <v>46302</v>
       </c>
       <c r="C126" t="n">
-        <v>1019</v>
+        <v>775</v>
       </c>
     </row>
     <row r="127">
@@ -2084,7 +2084,7 @@
         <v>46303</v>
       </c>
       <c r="C127" t="n">
-        <v>900</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="128">
@@ -2097,7 +2097,7 @@
         <v>46304</v>
       </c>
       <c r="C128" t="n">
-        <v>1208</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="129">
@@ -2110,7 +2110,7 @@
         <v>46305</v>
       </c>
       <c r="C129" t="n">
-        <v>937</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="130">
@@ -2123,7 +2123,7 @@
         <v>46307</v>
       </c>
       <c r="C130" t="n">
-        <v>1084</v>
+        <v>812</v>
       </c>
     </row>
     <row r="131">
@@ -2136,7 +2136,7 @@
         <v>46308</v>
       </c>
       <c r="C131" t="n">
-        <v>724</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="132">
@@ -2149,7 +2149,7 @@
         <v>46309</v>
       </c>
       <c r="C132" t="n">
-        <v>883</v>
+        <v>902</v>
       </c>
     </row>
     <row r="133">
@@ -2162,7 +2162,7 @@
         <v>46310</v>
       </c>
       <c r="C133" t="n">
-        <v>943</v>
+        <v>928</v>
       </c>
     </row>
     <row r="134">
@@ -2175,7 +2175,7 @@
         <v>46311</v>
       </c>
       <c r="C134" t="n">
-        <v>1135</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="135">
@@ -2188,7 +2188,7 @@
         <v>46312</v>
       </c>
       <c r="C135" t="n">
-        <v>673</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="136">
@@ -2201,7 +2201,7 @@
         <v>46314</v>
       </c>
       <c r="C136" t="n">
-        <v>1033</v>
+        <v>997</v>
       </c>
     </row>
     <row r="137">
@@ -2214,7 +2214,7 @@
         <v>46315</v>
       </c>
       <c r="C137" t="n">
-        <v>979</v>
+        <v>793</v>
       </c>
     </row>
     <row r="138">
@@ -2227,7 +2227,7 @@
         <v>46316</v>
       </c>
       <c r="C138" t="n">
-        <v>1107</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="139">
@@ -2240,7 +2240,7 @@
         <v>46317</v>
       </c>
       <c r="C139" t="n">
-        <v>996</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="140">
@@ -2253,7 +2253,7 @@
         <v>46318</v>
       </c>
       <c r="C140" t="n">
-        <v>907</v>
+        <v>965</v>
       </c>
     </row>
     <row r="141">
@@ -2266,7 +2266,7 @@
         <v>46319</v>
       </c>
       <c r="C141" t="n">
-        <v>829</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="142">
@@ -2279,7 +2279,7 @@
         <v>46321</v>
       </c>
       <c r="C142" t="n">
-        <v>731</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="143">
@@ -2292,7 +2292,7 @@
         <v>46322</v>
       </c>
       <c r="C143" t="n">
-        <v>926</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="144">
@@ -2305,7 +2305,7 @@
         <v>46323</v>
       </c>
       <c r="C144" t="n">
-        <v>874</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="145">
@@ -2318,7 +2318,7 @@
         <v>46324</v>
       </c>
       <c r="C145" t="n">
-        <v>1172</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="146">
@@ -2331,7 +2331,7 @@
         <v>46325</v>
       </c>
       <c r="C146" t="n">
-        <v>817</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="147">
@@ -2344,7 +2344,7 @@
         <v>46326</v>
       </c>
       <c r="C147" t="n">
-        <v>943</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="148">
@@ -2357,7 +2357,7 @@
         <v>46328</v>
       </c>
       <c r="C148" t="n">
-        <v>688</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="149">
@@ -2370,7 +2370,7 @@
         <v>46329</v>
       </c>
       <c r="C149" t="n">
-        <v>846</v>
+        <v>656</v>
       </c>
     </row>
     <row r="150">
@@ -2383,7 +2383,7 @@
         <v>46330</v>
       </c>
       <c r="C150" t="n">
-        <v>935</v>
+        <v>757</v>
       </c>
     </row>
     <row r="151">
@@ -2396,7 +2396,7 @@
         <v>46331</v>
       </c>
       <c r="C151" t="n">
-        <v>1011</v>
+        <v>642</v>
       </c>
     </row>
     <row r="152">
@@ -2409,7 +2409,7 @@
         <v>46332</v>
       </c>
       <c r="C152" t="n">
-        <v>1095</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="153">
@@ -2422,7 +2422,7 @@
         <v>46333</v>
       </c>
       <c r="C153" t="n">
-        <v>894</v>
+        <v>745</v>
       </c>
     </row>
     <row r="154">
@@ -2435,7 +2435,7 @@
         <v>46335</v>
       </c>
       <c r="C154" t="n">
-        <v>749</v>
+        <v>884</v>
       </c>
     </row>
     <row r="155">
@@ -2448,7 +2448,7 @@
         <v>46336</v>
       </c>
       <c r="C155" t="n">
-        <v>961</v>
+        <v>908</v>
       </c>
     </row>
     <row r="156">
@@ -2461,7 +2461,7 @@
         <v>46337</v>
       </c>
       <c r="C156" t="n">
-        <v>969</v>
+        <v>810</v>
       </c>
     </row>
     <row r="157">
@@ -2474,7 +2474,7 @@
         <v>46338</v>
       </c>
       <c r="C157" t="n">
-        <v>966</v>
+        <v>938</v>
       </c>
     </row>
     <row r="158">
@@ -2487,7 +2487,7 @@
         <v>46339</v>
       </c>
       <c r="C158" t="n">
-        <v>805</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="159">
@@ -2500,7 +2500,7 @@
         <v>46340</v>
       </c>
       <c r="C159" t="n">
-        <v>1053</v>
+        <v>914</v>
       </c>
     </row>
     <row r="160">
@@ -2513,7 +2513,7 @@
         <v>46342</v>
       </c>
       <c r="C160" t="n">
-        <v>911</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="161">
@@ -2526,7 +2526,7 @@
         <v>46343</v>
       </c>
       <c r="C161" t="n">
-        <v>994</v>
+        <v>886</v>
       </c>
     </row>
     <row r="162">
@@ -2539,7 +2539,7 @@
         <v>46344</v>
       </c>
       <c r="C162" t="n">
-        <v>1071</v>
+        <v>731</v>
       </c>
     </row>
     <row r="163">
@@ -2552,7 +2552,7 @@
         <v>46345</v>
       </c>
       <c r="C163" t="n">
-        <v>982</v>
+        <v>817</v>
       </c>
     </row>
     <row r="164">
@@ -2565,7 +2565,7 @@
         <v>46346</v>
       </c>
       <c r="C164" t="n">
-        <v>938</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="165">
@@ -2578,7 +2578,7 @@
         <v>46347</v>
       </c>
       <c r="C165" t="n">
-        <v>1190</v>
+        <v>667</v>
       </c>
     </row>
     <row r="166">
@@ -2591,7 +2591,7 @@
         <v>46349</v>
       </c>
       <c r="C166" t="n">
-        <v>932</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="167">
@@ -2604,7 +2604,7 @@
         <v>46350</v>
       </c>
       <c r="C167" t="n">
-        <v>860</v>
+        <v>989</v>
       </c>
     </row>
     <row r="168">
@@ -2617,7 +2617,7 @@
         <v>46351</v>
       </c>
       <c r="C168" t="n">
-        <v>915</v>
+        <v>899</v>
       </c>
     </row>
     <row r="169">
@@ -2630,7 +2630,7 @@
         <v>46352</v>
       </c>
       <c r="C169" t="n">
-        <v>1100</v>
+        <v>994</v>
       </c>
     </row>
     <row r="170">
@@ -2643,7 +2643,7 @@
         <v>46353</v>
       </c>
       <c r="C170" t="n">
-        <v>916</v>
+        <v>922</v>
       </c>
     </row>
     <row r="171">
@@ -2656,7 +2656,7 @@
         <v>46354</v>
       </c>
       <c r="C171" t="n">
-        <v>970</v>
+        <v>740</v>
       </c>
     </row>
     <row r="172">
@@ -2669,7 +2669,7 @@
         <v>46356</v>
       </c>
       <c r="C172" t="n">
-        <v>1061</v>
+        <v>815</v>
       </c>
     </row>
     <row r="173">
@@ -2682,7 +2682,7 @@
         <v>46357</v>
       </c>
       <c r="C173" t="n">
-        <v>830</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="174">
@@ -2695,7 +2695,7 @@
         <v>46358</v>
       </c>
       <c r="C174" t="n">
-        <v>666</v>
+        <v>807</v>
       </c>
     </row>
     <row r="175">
@@ -2708,7 +2708,7 @@
         <v>46359</v>
       </c>
       <c r="C175" t="n">
-        <v>940</v>
+        <v>788</v>
       </c>
     </row>
     <row r="176">
@@ -2721,7 +2721,7 @@
         <v>46360</v>
       </c>
       <c r="C176" t="n">
-        <v>931</v>
+        <v>794</v>
       </c>
     </row>
     <row r="177">
@@ -2734,7 +2734,7 @@
         <v>46361</v>
       </c>
       <c r="C177" t="n">
-        <v>817</v>
+        <v>694</v>
       </c>
     </row>
     <row r="178">
@@ -2747,7 +2747,7 @@
         <v>46363</v>
       </c>
       <c r="C178" t="n">
-        <v>1017</v>
+        <v>745</v>
       </c>
     </row>
     <row r="179">
@@ -2760,7 +2760,7 @@
         <v>46364</v>
       </c>
       <c r="C179" t="n">
-        <v>982</v>
+        <v>962</v>
       </c>
     </row>
     <row r="180">
@@ -2773,7 +2773,7 @@
         <v>46365</v>
       </c>
       <c r="C180" t="n">
-        <v>765</v>
+        <v>578</v>
       </c>
     </row>
     <row r="181">
@@ -2786,7 +2786,7 @@
         <v>46366</v>
       </c>
       <c r="C181" t="n">
-        <v>969</v>
+        <v>941</v>
       </c>
     </row>
     <row r="182">
@@ -2799,7 +2799,7 @@
         <v>46297</v>
       </c>
       <c r="C182" t="n">
-        <v>485</v>
+        <v>440</v>
       </c>
     </row>
     <row r="183">
@@ -2812,7 +2812,7 @@
         <v>46298</v>
       </c>
       <c r="C183" t="n">
-        <v>388</v>
+        <v>484</v>
       </c>
     </row>
     <row r="184">
@@ -2825,7 +2825,7 @@
         <v>46300</v>
       </c>
       <c r="C184" t="n">
-        <v>533</v>
+        <v>564</v>
       </c>
     </row>
     <row r="185">
@@ -2838,7 +2838,7 @@
         <v>46301</v>
       </c>
       <c r="C185" t="n">
-        <v>496</v>
+        <v>500</v>
       </c>
     </row>
     <row r="186">
@@ -2851,7 +2851,7 @@
         <v>46302</v>
       </c>
       <c r="C186" t="n">
-        <v>444</v>
+        <v>476</v>
       </c>
     </row>
     <row r="187">
@@ -2864,7 +2864,7 @@
         <v>46303</v>
       </c>
       <c r="C187" t="n">
-        <v>539</v>
+        <v>425</v>
       </c>
     </row>
     <row r="188">
@@ -2877,7 +2877,7 @@
         <v>46304</v>
       </c>
       <c r="C188" t="n">
-        <v>536</v>
+        <v>476</v>
       </c>
     </row>
     <row r="189">
@@ -2890,7 +2890,7 @@
         <v>46305</v>
       </c>
       <c r="C189" t="n">
-        <v>456</v>
+        <v>576</v>
       </c>
     </row>
     <row r="190">
@@ -2903,7 +2903,7 @@
         <v>46307</v>
       </c>
       <c r="C190" t="n">
-        <v>530</v>
+        <v>433</v>
       </c>
     </row>
     <row r="191">
@@ -2916,7 +2916,7 @@
         <v>46308</v>
       </c>
       <c r="C191" t="n">
-        <v>576</v>
+        <v>445</v>
       </c>
     </row>
     <row r="192">
@@ -2929,7 +2929,7 @@
         <v>46309</v>
       </c>
       <c r="C192" t="n">
-        <v>446</v>
+        <v>700</v>
       </c>
     </row>
     <row r="193">
@@ -2942,7 +2942,7 @@
         <v>46310</v>
       </c>
       <c r="C193" t="n">
-        <v>528</v>
+        <v>585</v>
       </c>
     </row>
     <row r="194">
@@ -2955,7 +2955,7 @@
         <v>46311</v>
       </c>
       <c r="C194" t="n">
-        <v>500</v>
+        <v>556</v>
       </c>
     </row>
     <row r="195">
@@ -2968,7 +2968,7 @@
         <v>46312</v>
       </c>
       <c r="C195" t="n">
-        <v>669</v>
+        <v>299</v>
       </c>
     </row>
     <row r="196">
@@ -2981,7 +2981,7 @@
         <v>46314</v>
       </c>
       <c r="C196" t="n">
-        <v>360</v>
+        <v>540</v>
       </c>
     </row>
     <row r="197">
@@ -2994,7 +2994,7 @@
         <v>46315</v>
       </c>
       <c r="C197" t="n">
-        <v>552</v>
+        <v>629</v>
       </c>
     </row>
     <row r="198">
@@ -3007,7 +3007,7 @@
         <v>46316</v>
       </c>
       <c r="C198" t="n">
-        <v>477</v>
+        <v>528</v>
       </c>
     </row>
     <row r="199">
@@ -3020,7 +3020,7 @@
         <v>46317</v>
       </c>
       <c r="C199" t="n">
-        <v>492</v>
+        <v>502</v>
       </c>
     </row>
     <row r="200">
@@ -3033,7 +3033,7 @@
         <v>46318</v>
       </c>
       <c r="C200" t="n">
-        <v>642</v>
+        <v>536</v>
       </c>
     </row>
     <row r="201">
@@ -3046,7 +3046,7 @@
         <v>46319</v>
       </c>
       <c r="C201" t="n">
-        <v>499</v>
+        <v>353</v>
       </c>
     </row>
     <row r="202">
@@ -3059,7 +3059,7 @@
         <v>46321</v>
       </c>
       <c r="C202" t="n">
-        <v>668</v>
+        <v>524</v>
       </c>
     </row>
     <row r="203">
@@ -3072,7 +3072,7 @@
         <v>46322</v>
       </c>
       <c r="C203" t="n">
-        <v>466</v>
+        <v>452</v>
       </c>
     </row>
     <row r="204">
@@ -3085,7 +3085,7 @@
         <v>46323</v>
       </c>
       <c r="C204" t="n">
-        <v>526</v>
+        <v>592</v>
       </c>
     </row>
     <row r="205">
@@ -3098,7 +3098,7 @@
         <v>46324</v>
       </c>
       <c r="C205" t="n">
-        <v>463</v>
+        <v>634</v>
       </c>
     </row>
     <row r="206">
@@ -3111,7 +3111,7 @@
         <v>46325</v>
       </c>
       <c r="C206" t="n">
-        <v>448</v>
+        <v>393</v>
       </c>
     </row>
     <row r="207">
@@ -3124,7 +3124,7 @@
         <v>46326</v>
       </c>
       <c r="C207" t="n">
-        <v>504</v>
+        <v>450</v>
       </c>
     </row>
     <row r="208">
@@ -3137,7 +3137,7 @@
         <v>46328</v>
       </c>
       <c r="C208" t="n">
-        <v>478</v>
+        <v>520</v>
       </c>
     </row>
     <row r="209">
@@ -3150,7 +3150,7 @@
         <v>46329</v>
       </c>
       <c r="C209" t="n">
-        <v>515</v>
+        <v>466</v>
       </c>
     </row>
     <row r="210">
@@ -3163,7 +3163,7 @@
         <v>46330</v>
       </c>
       <c r="C210" t="n">
-        <v>342</v>
+        <v>432</v>
       </c>
     </row>
     <row r="211">
@@ -3176,7 +3176,7 @@
         <v>46331</v>
       </c>
       <c r="C211" t="n">
-        <v>650</v>
+        <v>656</v>
       </c>
     </row>
     <row r="212">
@@ -3189,7 +3189,7 @@
         <v>46332</v>
       </c>
       <c r="C212" t="n">
-        <v>487</v>
+        <v>577</v>
       </c>
     </row>
     <row r="213">
@@ -3202,7 +3202,7 @@
         <v>46333</v>
       </c>
       <c r="C213" t="n">
-        <v>630</v>
+        <v>406</v>
       </c>
     </row>
     <row r="214">
@@ -3215,7 +3215,7 @@
         <v>46335</v>
       </c>
       <c r="C214" t="n">
-        <v>424</v>
+        <v>627</v>
       </c>
     </row>
     <row r="215">
@@ -3228,7 +3228,7 @@
         <v>46336</v>
       </c>
       <c r="C215" t="n">
-        <v>521</v>
+        <v>585</v>
       </c>
     </row>
     <row r="216">
@@ -3241,7 +3241,7 @@
         <v>46337</v>
       </c>
       <c r="C216" t="n">
-        <v>737</v>
+        <v>640</v>
       </c>
     </row>
     <row r="217">
@@ -3254,7 +3254,7 @@
         <v>46338</v>
       </c>
       <c r="C217" t="n">
-        <v>434</v>
+        <v>567</v>
       </c>
     </row>
     <row r="218">
@@ -3267,7 +3267,7 @@
         <v>46339</v>
       </c>
       <c r="C218" t="n">
-        <v>387</v>
+        <v>431</v>
       </c>
     </row>
     <row r="219">
@@ -3280,7 +3280,7 @@
         <v>46340</v>
       </c>
       <c r="C219" t="n">
-        <v>459</v>
+        <v>515</v>
       </c>
     </row>
     <row r="220">
@@ -3293,7 +3293,7 @@
         <v>46342</v>
       </c>
       <c r="C220" t="n">
-        <v>535</v>
+        <v>440</v>
       </c>
     </row>
     <row r="221">
@@ -3306,7 +3306,7 @@
         <v>46343</v>
       </c>
       <c r="C221" t="n">
-        <v>552</v>
+        <v>497</v>
       </c>
     </row>
     <row r="222">
@@ -3319,7 +3319,7 @@
         <v>46344</v>
       </c>
       <c r="C222" t="n">
-        <v>596</v>
+        <v>542</v>
       </c>
     </row>
     <row r="223">
@@ -3332,7 +3332,7 @@
         <v>46345</v>
       </c>
       <c r="C223" t="n">
-        <v>480</v>
+        <v>450</v>
       </c>
     </row>
     <row r="224">
@@ -3345,7 +3345,7 @@
         <v>46346</v>
       </c>
       <c r="C224" t="n">
-        <v>379</v>
+        <v>481</v>
       </c>
     </row>
     <row r="225">
@@ -3358,7 +3358,7 @@
         <v>46347</v>
       </c>
       <c r="C225" t="n">
-        <v>467</v>
+        <v>539</v>
       </c>
     </row>
     <row r="226">
@@ -3371,7 +3371,7 @@
         <v>46349</v>
       </c>
       <c r="C226" t="n">
-        <v>593</v>
+        <v>556</v>
       </c>
     </row>
     <row r="227">
@@ -3384,7 +3384,7 @@
         <v>46350</v>
       </c>
       <c r="C227" t="n">
-        <v>534</v>
+        <v>516</v>
       </c>
     </row>
     <row r="228">
@@ -3397,7 +3397,7 @@
         <v>46351</v>
       </c>
       <c r="C228" t="n">
-        <v>353</v>
+        <v>467</v>
       </c>
     </row>
     <row r="229">
@@ -3410,7 +3410,7 @@
         <v>46352</v>
       </c>
       <c r="C229" t="n">
-        <v>497</v>
+        <v>554</v>
       </c>
     </row>
     <row r="230">
@@ -3423,7 +3423,7 @@
         <v>46353</v>
       </c>
       <c r="C230" t="n">
-        <v>604</v>
+        <v>493</v>
       </c>
     </row>
     <row r="231">
@@ -3436,7 +3436,7 @@
         <v>46354</v>
       </c>
       <c r="C231" t="n">
-        <v>659</v>
+        <v>432</v>
       </c>
     </row>
     <row r="232">
@@ -3449,7 +3449,7 @@
         <v>46356</v>
       </c>
       <c r="C232" t="n">
-        <v>542</v>
+        <v>508</v>
       </c>
     </row>
     <row r="233">
@@ -3462,7 +3462,7 @@
         <v>46357</v>
       </c>
       <c r="C233" t="n">
-        <v>523</v>
+        <v>493</v>
       </c>
     </row>
     <row r="234">
@@ -3475,7 +3475,7 @@
         <v>46358</v>
       </c>
       <c r="C234" t="n">
-        <v>406</v>
+        <v>515</v>
       </c>
     </row>
     <row r="235">
@@ -3488,7 +3488,7 @@
         <v>46359</v>
       </c>
       <c r="C235" t="n">
-        <v>436</v>
+        <v>505</v>
       </c>
     </row>
     <row r="236">
@@ -3501,7 +3501,7 @@
         <v>46360</v>
       </c>
       <c r="C236" t="n">
-        <v>503</v>
+        <v>521</v>
       </c>
     </row>
     <row r="237">
@@ -3514,7 +3514,7 @@
         <v>46361</v>
       </c>
       <c r="C237" t="n">
-        <v>537</v>
+        <v>492</v>
       </c>
     </row>
     <row r="238">
@@ -3527,7 +3527,7 @@
         <v>46363</v>
       </c>
       <c r="C238" t="n">
-        <v>543</v>
+        <v>534</v>
       </c>
     </row>
     <row r="239">
@@ -3540,7 +3540,7 @@
         <v>46364</v>
       </c>
       <c r="C239" t="n">
-        <v>464</v>
+        <v>581</v>
       </c>
     </row>
     <row r="240">
@@ -3553,7 +3553,7 @@
         <v>46365</v>
       </c>
       <c r="C240" t="n">
-        <v>413</v>
+        <v>536</v>
       </c>
     </row>
     <row r="241">
@@ -3566,7 +3566,7 @@
         <v>46366</v>
       </c>
       <c r="C241" t="n">
-        <v>441</v>
+        <v>487</v>
       </c>
     </row>
     <row r="242">
@@ -3579,7 +3579,7 @@
         <v>46297</v>
       </c>
       <c r="C242" t="n">
-        <v>289</v>
+        <v>341</v>
       </c>
     </row>
     <row r="243">
@@ -3592,7 +3592,7 @@
         <v>46298</v>
       </c>
       <c r="C243" t="n">
-        <v>383</v>
+        <v>478</v>
       </c>
     </row>
     <row r="244">
@@ -3605,7 +3605,7 @@
         <v>46300</v>
       </c>
       <c r="C244" t="n">
-        <v>228</v>
+        <v>340</v>
       </c>
     </row>
     <row r="245">
@@ -3618,7 +3618,7 @@
         <v>46301</v>
       </c>
       <c r="C245" t="n">
-        <v>332</v>
+        <v>354</v>
       </c>
     </row>
     <row r="246">
@@ -3631,7 +3631,7 @@
         <v>46302</v>
       </c>
       <c r="C246" t="n">
-        <v>373</v>
+        <v>491</v>
       </c>
     </row>
     <row r="247">
@@ -3644,7 +3644,7 @@
         <v>46303</v>
       </c>
       <c r="C247" t="n">
-        <v>429</v>
+        <v>326</v>
       </c>
     </row>
     <row r="248">
@@ -3657,7 +3657,7 @@
         <v>46304</v>
       </c>
       <c r="C248" t="n">
-        <v>353</v>
+        <v>390</v>
       </c>
     </row>
     <row r="249">
@@ -3670,7 +3670,7 @@
         <v>46305</v>
       </c>
       <c r="C249" t="n">
-        <v>402</v>
+        <v>394</v>
       </c>
     </row>
     <row r="250">
@@ -3683,7 +3683,7 @@
         <v>46307</v>
       </c>
       <c r="C250" t="n">
-        <v>329</v>
+        <v>291</v>
       </c>
     </row>
     <row r="251">
@@ -3696,7 +3696,7 @@
         <v>46308</v>
       </c>
       <c r="C251" t="n">
-        <v>310</v>
+        <v>365</v>
       </c>
     </row>
     <row r="252">
@@ -3709,7 +3709,7 @@
         <v>46309</v>
       </c>
       <c r="C252" t="n">
-        <v>314</v>
+        <v>371</v>
       </c>
     </row>
     <row r="253">
@@ -3722,7 +3722,7 @@
         <v>46310</v>
       </c>
       <c r="C253" t="n">
-        <v>430</v>
+        <v>407</v>
       </c>
     </row>
     <row r="254">
@@ -3735,7 +3735,7 @@
         <v>46311</v>
       </c>
       <c r="C254" t="n">
-        <v>402</v>
+        <v>396</v>
       </c>
     </row>
     <row r="255">
@@ -3748,7 +3748,7 @@
         <v>46312</v>
       </c>
       <c r="C255" t="n">
-        <v>375</v>
+        <v>355</v>
       </c>
     </row>
     <row r="256">
@@ -3761,7 +3761,7 @@
         <v>46314</v>
       </c>
       <c r="C256" t="n">
-        <v>524</v>
+        <v>379</v>
       </c>
     </row>
     <row r="257">
@@ -3774,7 +3774,7 @@
         <v>46315</v>
       </c>
       <c r="C257" t="n">
-        <v>348</v>
+        <v>357</v>
       </c>
     </row>
     <row r="258">
@@ -3787,7 +3787,7 @@
         <v>46316</v>
       </c>
       <c r="C258" t="n">
-        <v>382</v>
+        <v>350</v>
       </c>
     </row>
     <row r="259">
@@ -3800,7 +3800,7 @@
         <v>46317</v>
       </c>
       <c r="C259" t="n">
-        <v>366</v>
+        <v>336</v>
       </c>
     </row>
     <row r="260">
@@ -3813,7 +3813,7 @@
         <v>46318</v>
       </c>
       <c r="C260" t="n">
-        <v>338</v>
+        <v>383</v>
       </c>
     </row>
     <row r="261">
@@ -3826,7 +3826,7 @@
         <v>46319</v>
       </c>
       <c r="C261" t="n">
-        <v>471</v>
+        <v>293</v>
       </c>
     </row>
     <row r="262">
@@ -3839,7 +3839,7 @@
         <v>46321</v>
       </c>
       <c r="C262" t="n">
-        <v>429</v>
+        <v>352</v>
       </c>
     </row>
     <row r="263">
@@ -3852,7 +3852,7 @@
         <v>46322</v>
       </c>
       <c r="C263" t="n">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="264">
@@ -3865,7 +3865,7 @@
         <v>46323</v>
       </c>
       <c r="C264" t="n">
-        <v>329</v>
+        <v>321</v>
       </c>
     </row>
     <row r="265">
@@ -3878,7 +3878,7 @@
         <v>46324</v>
       </c>
       <c r="C265" t="n">
-        <v>372</v>
+        <v>245</v>
       </c>
     </row>
     <row r="266">
@@ -3891,7 +3891,7 @@
         <v>46325</v>
       </c>
       <c r="C266" t="n">
-        <v>391</v>
+        <v>308</v>
       </c>
     </row>
     <row r="267">
@@ -3904,7 +3904,7 @@
         <v>46326</v>
       </c>
       <c r="C267" t="n">
-        <v>279</v>
+        <v>374</v>
       </c>
     </row>
     <row r="268">
@@ -3917,7 +3917,7 @@
         <v>46328</v>
       </c>
       <c r="C268" t="n">
-        <v>231</v>
+        <v>351</v>
       </c>
     </row>
     <row r="269">
@@ -3930,7 +3930,7 @@
         <v>46329</v>
       </c>
       <c r="C269" t="n">
-        <v>249</v>
+        <v>338</v>
       </c>
     </row>
     <row r="270">
@@ -3943,7 +3943,7 @@
         <v>46330</v>
       </c>
       <c r="C270" t="n">
-        <v>346</v>
+        <v>280</v>
       </c>
     </row>
     <row r="271">
@@ -3956,7 +3956,7 @@
         <v>46331</v>
       </c>
       <c r="C271" t="n">
-        <v>344</v>
+        <v>445</v>
       </c>
     </row>
     <row r="272">
@@ -3969,7 +3969,7 @@
         <v>46332</v>
       </c>
       <c r="C272" t="n">
-        <v>368</v>
+        <v>221</v>
       </c>
     </row>
     <row r="273">
@@ -3982,7 +3982,7 @@
         <v>46333</v>
       </c>
       <c r="C273" t="n">
-        <v>309</v>
+        <v>243</v>
       </c>
     </row>
     <row r="274">
@@ -3995,7 +3995,7 @@
         <v>46335</v>
       </c>
       <c r="C274" t="n">
-        <v>285</v>
+        <v>204</v>
       </c>
     </row>
     <row r="275">
@@ -4008,7 +4008,7 @@
         <v>46336</v>
       </c>
       <c r="C275" t="n">
-        <v>243</v>
+        <v>155</v>
       </c>
     </row>
     <row r="276">
@@ -4021,7 +4021,7 @@
         <v>46337</v>
       </c>
       <c r="C276" t="n">
-        <v>367</v>
+        <v>239</v>
       </c>
     </row>
     <row r="277">
@@ -4034,7 +4034,7 @@
         <v>46338</v>
       </c>
       <c r="C277" t="n">
-        <v>369</v>
+        <v>239</v>
       </c>
     </row>
     <row r="278">
@@ -4047,7 +4047,7 @@
         <v>46339</v>
       </c>
       <c r="C278" t="n">
-        <v>402</v>
+        <v>149</v>
       </c>
     </row>
     <row r="279">
@@ -4060,7 +4060,7 @@
         <v>46340</v>
       </c>
       <c r="C279" t="n">
-        <v>391</v>
+        <v>205</v>
       </c>
     </row>
     <row r="280">
@@ -4073,7 +4073,7 @@
         <v>46342</v>
       </c>
       <c r="C280" t="n">
-        <v>339</v>
+        <v>155</v>
       </c>
     </row>
     <row r="281">
@@ -4086,7 +4086,7 @@
         <v>46343</v>
       </c>
       <c r="C281" t="n">
-        <v>420</v>
+        <v>150</v>
       </c>
     </row>
     <row r="282">
@@ -4099,7 +4099,7 @@
         <v>46344</v>
       </c>
       <c r="C282" t="n">
-        <v>342</v>
+        <v>173</v>
       </c>
     </row>
     <row r="283">
@@ -4112,7 +4112,7 @@
         <v>46345</v>
       </c>
       <c r="C283" t="n">
-        <v>315</v>
+        <v>186</v>
       </c>
     </row>
     <row r="284">
@@ -4125,7 +4125,7 @@
         <v>46346</v>
       </c>
       <c r="C284" t="n">
-        <v>322</v>
+        <v>162</v>
       </c>
     </row>
     <row r="285">
@@ -4138,7 +4138,7 @@
         <v>46347</v>
       </c>
       <c r="C285" t="n">
-        <v>319</v>
+        <v>212</v>
       </c>
     </row>
     <row r="286">
@@ -4151,7 +4151,7 @@
         <v>46349</v>
       </c>
       <c r="C286" t="n">
-        <v>236</v>
+        <v>226</v>
       </c>
     </row>
     <row r="287">
@@ -4164,7 +4164,7 @@
         <v>46350</v>
       </c>
       <c r="C287" t="n">
-        <v>358</v>
+        <v>236</v>
       </c>
     </row>
     <row r="288">
@@ -4177,7 +4177,7 @@
         <v>46351</v>
       </c>
       <c r="C288" t="n">
-        <v>363</v>
+        <v>253</v>
       </c>
     </row>
     <row r="289">
@@ -4190,7 +4190,7 @@
         <v>46352</v>
       </c>
       <c r="C289" t="n">
-        <v>330</v>
+        <v>250</v>
       </c>
     </row>
     <row r="290">
@@ -4203,7 +4203,7 @@
         <v>46353</v>
       </c>
       <c r="C290" t="n">
-        <v>312</v>
+        <v>276</v>
       </c>
     </row>
     <row r="291">
@@ -4216,7 +4216,7 @@
         <v>46354</v>
       </c>
       <c r="C291" t="n">
-        <v>369</v>
+        <v>317</v>
       </c>
     </row>
     <row r="292">
@@ -4229,7 +4229,7 @@
         <v>46356</v>
       </c>
       <c r="C292" t="n">
-        <v>440</v>
+        <v>296</v>
       </c>
     </row>
     <row r="293">
@@ -4242,7 +4242,7 @@
         <v>46357</v>
       </c>
       <c r="C293" t="n">
-        <v>352</v>
+        <v>342</v>
       </c>
     </row>
     <row r="294">
@@ -4255,7 +4255,7 @@
         <v>46358</v>
       </c>
       <c r="C294" t="n">
-        <v>323</v>
+        <v>353</v>
       </c>
     </row>
     <row r="295">
@@ -4268,7 +4268,7 @@
         <v>46359</v>
       </c>
       <c r="C295" t="n">
-        <v>318</v>
+        <v>371</v>
       </c>
     </row>
     <row r="296">
@@ -4281,7 +4281,7 @@
         <v>46360</v>
       </c>
       <c r="C296" t="n">
-        <v>346</v>
+        <v>261</v>
       </c>
     </row>
     <row r="297">
@@ -4294,7 +4294,7 @@
         <v>46361</v>
       </c>
       <c r="C297" t="n">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="298">
@@ -4307,7 +4307,7 @@
         <v>46363</v>
       </c>
       <c r="C298" t="n">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="299">
@@ -4320,7 +4320,7 @@
         <v>46364</v>
       </c>
       <c r="C299" t="n">
-        <v>353</v>
+        <v>338</v>
       </c>
     </row>
     <row r="300">
@@ -4333,7 +4333,7 @@
         <v>46365</v>
       </c>
       <c r="C300" t="n">
-        <v>446</v>
+        <v>349</v>
       </c>
     </row>
     <row r="301">
@@ -4346,7 +4346,7 @@
         <v>46366</v>
       </c>
       <c r="C301" t="n">
-        <v>399</v>
+        <v>304</v>
       </c>
     </row>
     <row r="302">
@@ -4359,7 +4359,7 @@
         <v>46297</v>
       </c>
       <c r="C302" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="303">
@@ -4372,7 +4372,7 @@
         <v>46298</v>
       </c>
       <c r="C303" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="304">
@@ -4385,7 +4385,7 @@
         <v>46300</v>
       </c>
       <c r="C304" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="305">
@@ -4398,7 +4398,7 @@
         <v>46301</v>
       </c>
       <c r="C305" t="n">
-        <v>82</v>
+        <v>118</v>
       </c>
     </row>
     <row r="306">
@@ -4411,7 +4411,7 @@
         <v>46302</v>
       </c>
       <c r="C306" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="307">
@@ -4424,7 +4424,7 @@
         <v>46303</v>
       </c>
       <c r="C307" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="308">
@@ -4437,7 +4437,7 @@
         <v>46304</v>
       </c>
       <c r="C308" t="n">
-        <v>88</v>
+        <v>64</v>
       </c>
     </row>
     <row r="309">
@@ -4450,7 +4450,7 @@
         <v>46305</v>
       </c>
       <c r="C309" t="n">
-        <v>129</v>
+        <v>86</v>
       </c>
     </row>
     <row r="310">
@@ -4463,7 +4463,7 @@
         <v>46307</v>
       </c>
       <c r="C310" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="311">
@@ -4476,7 +4476,7 @@
         <v>46308</v>
       </c>
       <c r="C311" t="n">
-        <v>71</v>
+        <v>135</v>
       </c>
     </row>
     <row r="312">
@@ -4489,7 +4489,7 @@
         <v>46309</v>
       </c>
       <c r="C312" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="313">
@@ -4502,7 +4502,7 @@
         <v>46310</v>
       </c>
       <c r="C313" t="n">
-        <v>93</v>
+        <v>117</v>
       </c>
     </row>
     <row r="314">
@@ -4515,7 +4515,7 @@
         <v>46311</v>
       </c>
       <c r="C314" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="315">
@@ -4528,7 +4528,7 @@
         <v>46312</v>
       </c>
       <c r="C315" t="n">
-        <v>106</v>
+        <v>115</v>
       </c>
     </row>
     <row r="316">
@@ -4541,7 +4541,7 @@
         <v>46314</v>
       </c>
       <c r="C316" t="n">
-        <v>105</v>
+        <v>96</v>
       </c>
     </row>
     <row r="317">
@@ -4554,7 +4554,7 @@
         <v>46315</v>
       </c>
       <c r="C317" t="n">
-        <v>69</v>
+        <v>109</v>
       </c>
     </row>
     <row r="318">
@@ -4567,7 +4567,7 @@
         <v>46316</v>
       </c>
       <c r="C318" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="319">
@@ -4580,7 +4580,7 @@
         <v>46317</v>
       </c>
       <c r="C319" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="320">
@@ -4593,7 +4593,7 @@
         <v>46318</v>
       </c>
       <c r="C320" t="n">
-        <v>119</v>
+        <v>84</v>
       </c>
     </row>
     <row r="321">
@@ -4606,7 +4606,7 @@
         <v>46319</v>
       </c>
       <c r="C321" t="n">
-        <v>128</v>
+        <v>104</v>
       </c>
     </row>
     <row r="322">
@@ -4619,7 +4619,7 @@
         <v>46321</v>
       </c>
       <c r="C322" t="n">
-        <v>127</v>
+        <v>96</v>
       </c>
     </row>
     <row r="323">
@@ -4632,7 +4632,7 @@
         <v>46322</v>
       </c>
       <c r="C323" t="n">
-        <v>69</v>
+        <v>101</v>
       </c>
     </row>
     <row r="324">
@@ -4645,7 +4645,7 @@
         <v>46323</v>
       </c>
       <c r="C324" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="325">
@@ -4658,7 +4658,7 @@
         <v>46324</v>
       </c>
       <c r="C325" t="n">
-        <v>71</v>
+        <v>101</v>
       </c>
     </row>
     <row r="326">
@@ -4671,7 +4671,7 @@
         <v>46325</v>
       </c>
       <c r="C326" t="n">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="327">
@@ -4684,7 +4684,7 @@
         <v>46326</v>
       </c>
       <c r="C327" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="328">
@@ -4697,7 +4697,7 @@
         <v>46328</v>
       </c>
       <c r="C328" t="n">
-        <v>82</v>
+        <v>111</v>
       </c>
     </row>
     <row r="329">
@@ -4710,7 +4710,7 @@
         <v>46329</v>
       </c>
       <c r="C329" t="n">
-        <v>130</v>
+        <v>88</v>
       </c>
     </row>
     <row r="330">
@@ -4723,7 +4723,7 @@
         <v>46330</v>
       </c>
       <c r="C330" t="n">
-        <v>109</v>
+        <v>125</v>
       </c>
     </row>
     <row r="331">
@@ -4736,7 +4736,7 @@
         <v>46331</v>
       </c>
       <c r="C331" t="n">
-        <v>71</v>
+        <v>126</v>
       </c>
     </row>
     <row r="332">
@@ -4749,7 +4749,7 @@
         <v>46332</v>
       </c>
       <c r="C332" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="333">
@@ -4762,7 +4762,7 @@
         <v>46333</v>
       </c>
       <c r="C333" t="n">
-        <v>89</v>
+        <v>105</v>
       </c>
     </row>
     <row r="334">
@@ -4775,7 +4775,7 @@
         <v>46335</v>
       </c>
       <c r="C334" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
     </row>
     <row r="335">
@@ -4788,7 +4788,7 @@
         <v>46336</v>
       </c>
       <c r="C335" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="336">
@@ -4801,7 +4801,7 @@
         <v>46337</v>
       </c>
       <c r="C336" t="n">
-        <v>120</v>
+        <v>108</v>
       </c>
     </row>
     <row r="337">
@@ -4814,7 +4814,7 @@
         <v>46338</v>
       </c>
       <c r="C337" t="n">
-        <v>78</v>
+        <v>94</v>
       </c>
     </row>
     <row r="338">
@@ -4827,7 +4827,7 @@
         <v>46339</v>
       </c>
       <c r="C338" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
     </row>
     <row r="339">
@@ -4840,7 +4840,7 @@
         <v>46340</v>
       </c>
       <c r="C339" t="n">
-        <v>127</v>
+        <v>112</v>
       </c>
     </row>
     <row r="340">
@@ -4853,7 +4853,7 @@
         <v>46342</v>
       </c>
       <c r="C340" t="n">
-        <v>87</v>
+        <v>99</v>
       </c>
     </row>
     <row r="341">
@@ -4866,7 +4866,7 @@
         <v>46343</v>
       </c>
       <c r="C341" t="n">
-        <v>103</v>
+        <v>90</v>
       </c>
     </row>
     <row r="342">
@@ -4879,7 +4879,7 @@
         <v>46344</v>
       </c>
       <c r="C342" t="n">
-        <v>103</v>
+        <v>114</v>
       </c>
     </row>
     <row r="343">
@@ -4892,7 +4892,7 @@
         <v>46345</v>
       </c>
       <c r="C343" t="n">
-        <v>89</v>
+        <v>100</v>
       </c>
     </row>
     <row r="344">
@@ -4905,7 +4905,7 @@
         <v>46346</v>
       </c>
       <c r="C344" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="345">
@@ -4918,7 +4918,7 @@
         <v>46347</v>
       </c>
       <c r="C345" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
     </row>
     <row r="346">
@@ -4931,7 +4931,7 @@
         <v>46349</v>
       </c>
       <c r="C346" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="347">
@@ -4944,7 +4944,7 @@
         <v>46350</v>
       </c>
       <c r="C347" t="n">
-        <v>126</v>
+        <v>136</v>
       </c>
     </row>
     <row r="348">
@@ -4957,7 +4957,7 @@
         <v>46351</v>
       </c>
       <c r="C348" t="n">
-        <v>111</v>
+        <v>99</v>
       </c>
     </row>
     <row r="349">
@@ -4970,7 +4970,7 @@
         <v>46352</v>
       </c>
       <c r="C349" t="n">
-        <v>97</v>
+        <v>112</v>
       </c>
     </row>
     <row r="350">
@@ -4996,7 +4996,7 @@
         <v>46354</v>
       </c>
       <c r="C351" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="352">
@@ -5009,7 +5009,7 @@
         <v>46356</v>
       </c>
       <c r="C352" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
     </row>
     <row r="353">
@@ -5022,7 +5022,7 @@
         <v>46357</v>
       </c>
       <c r="C353" t="n">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="354">
@@ -5035,7 +5035,7 @@
         <v>46358</v>
       </c>
       <c r="C354" t="n">
-        <v>106</v>
+        <v>80</v>
       </c>
     </row>
     <row r="355">
@@ -5048,7 +5048,7 @@
         <v>46359</v>
       </c>
       <c r="C355" t="n">
-        <v>97</v>
+        <v>76</v>
       </c>
     </row>
     <row r="356">
@@ -5061,7 +5061,7 @@
         <v>46360</v>
       </c>
       <c r="C356" t="n">
-        <v>109</v>
+        <v>75</v>
       </c>
     </row>
     <row r="357">
@@ -5074,7 +5074,7 @@
         <v>46361</v>
       </c>
       <c r="C357" t="n">
-        <v>98</v>
+        <v>118</v>
       </c>
     </row>
     <row r="358">
@@ -5087,7 +5087,7 @@
         <v>46363</v>
       </c>
       <c r="C358" t="n">
-        <v>111</v>
+        <v>100</v>
       </c>
     </row>
     <row r="359">
@@ -5100,7 +5100,7 @@
         <v>46364</v>
       </c>
       <c r="C359" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="360">
@@ -5113,7 +5113,7 @@
         <v>46365</v>
       </c>
       <c r="C360" t="n">
-        <v>112</v>
+        <v>96</v>
       </c>
     </row>
     <row r="361">
@@ -5126,7 +5126,7 @@
         <v>46366</v>
       </c>
       <c r="C361" t="n">
-        <v>110</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>